<commit_message>
68_생산중량계산_JSP_MSSQL전환 ### Step 1: JSP MSSQL 전환
search_production_calc.jsp 를 CO_품목코드 기반으로 전환. PDA JSP 18개 전부 전환 완료.

- B_SUPPLIER_ITEM + S_BARCODE_INFO -> CO_품목코드 단일 (조인 소멸)
- ROWNUM = 1 -> SELECT TOP 1
- A.STATUS = 'Y' 삭제 (search_barcode_info.jsp 전례, 생산품상태는 '3' 계열로 대체 불가)
- qry_where 치환 2건 (a.PACKER_CODE -> SBI.패커코드, a.PACKER_PRODUCT_CODE -> SBI.ppCode)
- 회사코드 미추가 (앱 미전송, 하드코딩 JSP 0건)

앱 무수정. 출력 4개 컬럼 수/순서/구분자 유지.
앱 실제 포맷 호출 검증: HTTP 500 -> 200, 응답 1::5::2::KG (4개 컬럼 일치)

함께 수정
- PDA테스트문서.xlsx P-17: 존재하지 않는 "서버 전송" TC 를 실제 동작으로 교체
- 오류36: "미전환 별도 관리" 기록 해소 처리
- 일정 2026-09-27: 완료 작업 2건 추가, searchType별 데이터 실측치 갱신

Step 2(통합 테스트)는 ERP CO_품목코드 패커코드/ppCode 입력 후 진행.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/doc/테스트/PDA테스트문서.xlsx
+++ b/app/doc/테스트/PDA테스트문서.xlsx
@@ -1438,17 +1438,18 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>서버 전송</t>
+          <t>바코드정보 수신 서버 응답 확인</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>계근 완료 후 전송 수행</t>
+          <t>PACKER코드·PP코드 입력 후 [바코드정보 수신] 클릭 → Tomcat 로그 확인</t>
         </is>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>search_production_calc.jsp 로 전송되어 결과 확인</t>
+          <t>search_production_calc.jsp 응답이 WEIGHT_FROM::WEIGHT_TO::ZEROPOINT::BASEUNIT 4개 값으로 수신됨
+로그 ##serch_shipment query: 에 SBI.패커코드·SBI.ppCode 치환 확인</t>
         </is>
       </c>
       <c r="E22" s="22" t="inlineStr"/>
@@ -1461,7 +1462,7 @@
       <c r="H22" s="21" t="inlineStr"/>
       <c r="I22" s="22" t="inlineStr">
         <is>
-          <t>현 상태 유지 기능 - MSSQL 전환 보류 상태. 전송 가능 여부 먼저 확인</t>
+          <t>개발68 MSSQL 전환 완료(2026-09-27). 이 화면은 서버 전송 기능 없음 - 계근결과는 로컬 SQLite만 사용</t>
         </is>
       </c>
     </row>

</xml_diff>